<commit_message>
Actualización automática: datos al 2026-06-26
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-25)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-26)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AM4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AM5</f>
@@ -3158,7 +3158,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM2" t="n">
-        <v>217311612.51</v>
+        <v>216174403.99</v>
       </c>
     </row>
     <row r="3">
@@ -3264,7 +3264,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM3" t="n">
-        <v>680488357.37</v>
+        <v>680648576.01</v>
       </c>
     </row>
     <row r="4">
@@ -3497,7 +3497,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>217311612.51</v>
+        <v>216174403.99</v>
       </c>
     </row>
     <row r="12">
@@ -3516,7 +3516,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>680488357.37</v>
+        <v>680648576.01</v>
       </c>
     </row>
     <row r="13">
@@ -3886,7 +3886,7 @@
         <v>0.003951</v>
       </c>
       <c r="AM20" t="n">
-        <v>0.003024</v>
+        <v>0.003157</v>
       </c>
     </row>
     <row r="21">
@@ -3992,7 +3992,7 @@
         <v>-0.011932</v>
       </c>
       <c r="AM21" t="n">
-        <v>-0.001397</v>
+        <v>-0.001162</v>
       </c>
     </row>
     <row r="22">
@@ -4206,7 +4206,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-25) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-26) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-25)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-26)</t>
         </is>
       </c>
     </row>
@@ -5580,7 +5580,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-25) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-26) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5716,6 +5716,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46198</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.17526606</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>216174403.99</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1039.57713645</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>680648576.01</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1219.0985505</v>
@@ -44529,7 +44547,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-25)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-26)</t>
         </is>
       </c>
     </row>
@@ -44848,7 +44866,7 @@
         <v>1.17156713</v>
       </c>
       <c r="AM4" s="24" t="n">
-        <v>1.17511014</v>
+        <v>1.17526606</v>
       </c>
     </row>
     <row r="5">
@@ -44959,7 +44977,7 @@
         <v>1040.78664211</v>
       </c>
       <c r="AM5" s="24" t="n">
-        <v>1039.33242922</v>
+        <v>1039.57713645</v>
       </c>
     </row>
     <row r="6">
@@ -45317,7 +45335,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-25)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-06-25 (actualización 2026-06-26)</t>
         </is>
       </c>
     </row>
@@ -45636,7 +45654,7 @@
         <v>217688480.9</v>
       </c>
       <c r="AM4" s="25" t="n">
-        <v>217311612.51</v>
+        <v>216174403.99</v>
       </c>
     </row>
     <row r="5">
@@ -45747,7 +45765,7 @@
         <v>681440482.91</v>
       </c>
       <c r="AM5" s="25" t="n">
-        <v>680488357.37</v>
+        <v>680648576.01</v>
       </c>
     </row>
     <row r="6">
@@ -46077,7 +46095,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-06-25 (actualización 2026-06-25).</t>
+          <t>datos al 2026-06-25 (actualización 2026-06-26).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-07-05
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AN4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46206</v>
+        <v>46207</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AN5</f>
@@ -3166,7 +3166,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN2" t="n">
-        <v>229400158.58</v>
+        <v>229435263.52</v>
       </c>
     </row>
     <row r="3">
@@ -3275,7 +3275,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN3" t="n">
-        <v>681919832.73</v>
+        <v>682079981.83</v>
       </c>
     </row>
     <row r="4">
@@ -3520,7 +3520,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>229400158.58</v>
+        <v>229435263.52</v>
       </c>
     </row>
     <row r="12">
@@ -3539,7 +3539,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>681919832.73</v>
+        <v>682079981.83</v>
       </c>
     </row>
     <row r="13">
@@ -3917,7 +3917,7 @@
         <v>0.003825</v>
       </c>
       <c r="AN20" t="n">
-        <v>0.00041</v>
+        <v>0.0005419999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -4026,7 +4026,7 @@
         <v>-3e-06</v>
       </c>
       <c r="AN21" t="n">
-        <v>0.0007069999999999999</v>
+        <v>0.000942</v>
       </c>
     </row>
     <row r="22">
@@ -4252,7 +4252,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-04) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05)</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-04) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5833,6 +5833,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46207</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.17668648</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000132</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>229435263.52</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1041.76337001</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>682079981.83</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1220.97578907</v>
@@ -45178,7 +45196,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05)</t>
         </is>
       </c>
     </row>
@@ -45505,7 +45523,7 @@
         <v>1.17604869</v>
       </c>
       <c r="AN4" s="24" t="n">
-        <v>1.17653062</v>
+        <v>1.17668648</v>
       </c>
     </row>
     <row r="5">
@@ -45619,7 +45637,7 @@
         <v>1040.78324635</v>
       </c>
       <c r="AN5" s="24" t="n">
-        <v>1041.51876899</v>
+        <v>1041.76337001</v>
       </c>
     </row>
     <row r="6">
@@ -45990,7 +46008,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05)</t>
         </is>
       </c>
     </row>
@@ -46317,7 +46335,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN4" s="25" t="n">
-        <v>229400158.58</v>
+        <v>229435263.52</v>
       </c>
     </row>
     <row r="5">
@@ -46431,7 +46449,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN5" s="25" t="n">
-        <v>681919832.73</v>
+        <v>682079981.83</v>
       </c>
     </row>
     <row r="6">
@@ -46773,7 +46791,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-07-05 (actualización 2026-07-04).</t>
+          <t>datos al 2026-07-05 (actualización 2026-07-05).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-07-06
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-06)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AN4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46207</v>
+        <v>46208</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AN5</f>
@@ -3166,7 +3166,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN2" t="n">
-        <v>229435263.52</v>
+        <v>229463683.29</v>
       </c>
     </row>
     <row r="3">
@@ -3275,7 +3275,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN3" t="n">
-        <v>682079981.83</v>
+        <v>682240572.35</v>
       </c>
     </row>
     <row r="4">
@@ -3520,7 +3520,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>229435263.52</v>
+        <v>229463683.29</v>
       </c>
     </row>
     <row r="12">
@@ -3539,7 +3539,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>682079981.83</v>
+        <v>682240572.35</v>
       </c>
     </row>
     <row r="13">
@@ -3917,7 +3917,7 @@
         <v>0.003825</v>
       </c>
       <c r="AN20" t="n">
-        <v>0.0005419999999999999</v>
+        <v>0.000674</v>
       </c>
     </row>
     <row r="21">
@@ -4026,7 +4026,7 @@
         <v>-3e-06</v>
       </c>
       <c r="AN21" t="n">
-        <v>0.000942</v>
+        <v>0.001177</v>
       </c>
     </row>
     <row r="22">
@@ -4252,7 +4252,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-06) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-06)</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-06) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5792,6 +5792,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46208</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.17684183</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000132</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>229463683.29</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1042.00864524</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>682240572.35</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1221.13734042</v>
@@ -45196,7 +45214,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-06)</t>
         </is>
       </c>
     </row>
@@ -45523,7 +45541,7 @@
         <v>1.17604869</v>
       </c>
       <c r="AN4" s="24" t="n">
-        <v>1.17668648</v>
+        <v>1.17684183</v>
       </c>
     </row>
     <row r="5">
@@ -45637,7 +45655,7 @@
         <v>1040.78324635</v>
       </c>
       <c r="AN5" s="24" t="n">
-        <v>1041.76337001</v>
+        <v>1042.00864524</v>
       </c>
     </row>
     <row r="6">
@@ -46008,7 +46026,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-05 (actualización 2026-07-06)</t>
         </is>
       </c>
     </row>
@@ -46335,7 +46353,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN4" s="25" t="n">
-        <v>229435263.52</v>
+        <v>229463683.29</v>
       </c>
     </row>
     <row r="5">
@@ -46449,7 +46467,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN5" s="25" t="n">
-        <v>682079981.83</v>
+        <v>682240572.35</v>
       </c>
     </row>
     <row r="6">
@@ -46791,7 +46809,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-07-05 (actualización 2026-07-05).</t>
+          <t>datos al 2026-07-05 (actualización 2026-07-06).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-07-12
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-11)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AN4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46213</v>
+        <v>46214</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AN5</f>
@@ -3166,7 +3166,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN2" t="n">
-        <v>228346554.78</v>
+        <v>228379004.08</v>
       </c>
     </row>
     <row r="3">
@@ -3275,7 +3275,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN3" t="n">
-        <v>683042801.2</v>
+        <v>683202569.0599999</v>
       </c>
     </row>
     <row r="4">
@@ -3520,7 +3520,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>228346554.78</v>
+        <v>228379004.08</v>
       </c>
     </row>
     <row r="12">
@@ -3539,7 +3539,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>683042801.2</v>
+        <v>683202569.0599999</v>
       </c>
     </row>
     <row r="13">
@@ -3917,7 +3917,7 @@
         <v>0.003825</v>
       </c>
       <c r="AN20" t="n">
-        <v>0.001322</v>
+        <v>0.001455</v>
       </c>
     </row>
     <row r="21">
@@ -4026,7 +4026,7 @@
         <v>-3e-06</v>
       </c>
       <c r="AN21" t="n">
-        <v>0.002355</v>
+        <v>0.002589</v>
       </c>
     </row>
     <row r="22">
@@ -4252,7 +4252,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-11) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-11)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12)</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-11) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5833,6 +5833,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46214</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.17775981</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>228379004.08</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1043.47793471</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>683202569.0599999</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1222.10692098</v>
@@ -45591,7 +45609,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-11)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12)</t>
         </is>
       </c>
     </row>
@@ -45918,7 +45936,7 @@
         <v>1.17604869</v>
       </c>
       <c r="AN4" s="24" t="n">
-        <v>1.17760364</v>
+        <v>1.17775981</v>
       </c>
     </row>
     <row r="5">
@@ -46032,7 +46050,7 @@
         <v>1040.78324635</v>
       </c>
       <c r="AN5" s="24" t="n">
-        <v>1043.23391596</v>
+        <v>1043.47793471</v>
       </c>
     </row>
     <row r="6">
@@ -46403,7 +46421,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-11)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12)</t>
         </is>
       </c>
     </row>
@@ -46730,7 +46748,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN4" s="25" t="n">
-        <v>228346554.78</v>
+        <v>228379004.08</v>
       </c>
     </row>
     <row r="5">
@@ -46844,7 +46862,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN5" s="25" t="n">
-        <v>683042801.2</v>
+        <v>683202569.0599999</v>
       </c>
     </row>
     <row r="6">
@@ -47186,7 +47204,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-07-12 (actualización 2026-07-11).</t>
+          <t>datos al 2026-07-12 (actualización 2026-07-12).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-07-13
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-13)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AN4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46214</v>
+        <v>46215</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AN5</f>
@@ -3166,7 +3166,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN2" t="n">
-        <v>228379004.08</v>
+        <v>228415948.21</v>
       </c>
     </row>
     <row r="3">
@@ -3275,7 +3275,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN3" t="n">
-        <v>683202569.0599999</v>
+        <v>683363034.87</v>
       </c>
     </row>
     <row r="4">
@@ -3520,7 +3520,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>228379004.08</v>
+        <v>228415948.21</v>
       </c>
     </row>
     <row r="12">
@@ -3539,7 +3539,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>683202569.0599999</v>
+        <v>683363034.87</v>
       </c>
     </row>
     <row r="13">
@@ -3917,7 +3917,7 @@
         <v>0.003825</v>
       </c>
       <c r="AN20" t="n">
-        <v>0.001455</v>
+        <v>0.001588</v>
       </c>
     </row>
     <row r="21">
@@ -4026,7 +4026,7 @@
         <v>-3e-06</v>
       </c>
       <c r="AN21" t="n">
-        <v>0.002589</v>
+        <v>0.002825</v>
       </c>
     </row>
     <row r="22">
@@ -4252,7 +4252,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-13) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-13)</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-13) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5792,6 +5792,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46215</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.17791593</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>228415948.21</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1043.72301946</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>683363034.87</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1222.26853263</v>
@@ -45609,7 +45627,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-13)</t>
         </is>
       </c>
     </row>
@@ -45936,7 +45954,7 @@
         <v>1.17604869</v>
       </c>
       <c r="AN4" s="24" t="n">
-        <v>1.17775981</v>
+        <v>1.17791593</v>
       </c>
     </row>
     <row r="5">
@@ -46050,7 +46068,7 @@
         <v>1040.78324635</v>
       </c>
       <c r="AN5" s="24" t="n">
-        <v>1043.47793471</v>
+        <v>1043.72301946</v>
       </c>
     </row>
     <row r="6">
@@ -46421,7 +46439,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-12)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-12 (actualización 2026-07-13)</t>
         </is>
       </c>
     </row>
@@ -46748,7 +46766,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN4" s="25" t="n">
-        <v>228379004.08</v>
+        <v>228415948.21</v>
       </c>
     </row>
     <row r="5">
@@ -46862,7 +46880,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN5" s="25" t="n">
-        <v>683202569.0599999</v>
+        <v>683363034.87</v>
       </c>
     </row>
     <row r="6">
@@ -47204,7 +47222,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-07-12 (actualización 2026-07-12).</t>
+          <t>datos al 2026-07-12 (actualización 2026-07-13).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-07-19
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-18)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AN4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AN5</f>
@@ -3166,7 +3166,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN2" t="n">
-        <v>235895517.9</v>
+        <v>235930884.45</v>
       </c>
     </row>
     <row r="3">
@@ -3275,7 +3275,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN3" t="n">
-        <v>684166549.4299999</v>
+        <v>684327181.79</v>
       </c>
     </row>
     <row r="4">
@@ -3520,7 +3520,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>235895517.9</v>
+        <v>235930884.45</v>
       </c>
     </row>
     <row r="12">
@@ -3539,7 +3539,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>684166549.4299999</v>
+        <v>684327181.79</v>
       </c>
     </row>
     <row r="13">
@@ -3917,7 +3917,7 @@
         <v>0.003825</v>
       </c>
       <c r="AN20" t="n">
-        <v>0.002213</v>
+        <v>0.002344</v>
       </c>
     </row>
     <row r="21">
@@ -4026,7 +4026,7 @@
         <v>-3e-06</v>
       </c>
       <c r="AN21" t="n">
-        <v>0.004004</v>
+        <v>0.004239</v>
       </c>
     </row>
     <row r="22">
@@ -4252,7 +4252,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-18) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-18)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19)</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-18) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5833,6 +5833,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46221</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.17880488</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.00013</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>235930884.45</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1045.19559302</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>684327181.79</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1223.24984679</v>
@@ -45995,7 +46013,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-18)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19)</t>
         </is>
       </c>
     </row>
@@ -46322,7 +46340,7 @@
         <v>1.17604869</v>
       </c>
       <c r="AN4" s="24" t="n">
-        <v>1.1786514</v>
+        <v>1.17880488</v>
       </c>
     </row>
     <row r="5">
@@ -46436,7 +46454,7 @@
         <v>1040.78324635</v>
       </c>
       <c r="AN5" s="24" t="n">
-        <v>1044.95025389</v>
+        <v>1045.19559302</v>
       </c>
     </row>
     <row r="6">
@@ -46807,7 +46825,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-18)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19)</t>
         </is>
       </c>
     </row>
@@ -47134,7 +47152,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN4" s="25" t="n">
-        <v>235895517.9</v>
+        <v>235930884.45</v>
       </c>
     </row>
     <row r="5">
@@ -47248,7 +47266,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN5" s="25" t="n">
-        <v>684166549.4299999</v>
+        <v>684327181.79</v>
       </c>
     </row>
     <row r="6">
@@ -47590,7 +47608,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-07-19 (actualización 2026-07-18).</t>
+          <t>datos al 2026-07-19 (actualización 2026-07-19).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-07-20
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-20)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AN4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AN5</f>
@@ -3166,7 +3166,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN2" t="n">
-        <v>235930884.45</v>
+        <v>235975601.38</v>
       </c>
     </row>
     <row r="3">
@@ -3275,7 +3275,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN3" t="n">
-        <v>684327181.79</v>
+        <v>684487486.2</v>
       </c>
     </row>
     <row r="4">
@@ -3520,7 +3520,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>235930884.45</v>
+        <v>235975601.38</v>
       </c>
     </row>
     <row r="12">
@@ -3539,7 +3539,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>684327181.79</v>
+        <v>684487486.2</v>
       </c>
     </row>
     <row r="13">
@@ -3917,7 +3917,7 @@
         <v>0.003825</v>
       </c>
       <c r="AN20" t="n">
-        <v>0.002344</v>
+        <v>0.002475</v>
       </c>
     </row>
     <row r="21">
@@ -4026,7 +4026,7 @@
         <v>-3e-06</v>
       </c>
       <c r="AN21" t="n">
-        <v>0.004239</v>
+        <v>0.004475</v>
       </c>
     </row>
     <row r="22">
@@ -4252,7 +4252,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-20) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-20)</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-20) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5792,6 +5792,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46222</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.17895917</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000131</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>235975601.38</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1045.44043126</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>684487486.2</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1223.41726582</v>
@@ -46013,7 +46031,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-20)</t>
         </is>
       </c>
     </row>
@@ -46340,7 +46358,7 @@
         <v>1.17604869</v>
       </c>
       <c r="AN4" s="24" t="n">
-        <v>1.17880488</v>
+        <v>1.17895917</v>
       </c>
     </row>
     <row r="5">
@@ -46454,7 +46472,7 @@
         <v>1040.78324635</v>
       </c>
       <c r="AN5" s="24" t="n">
-        <v>1045.19559302</v>
+        <v>1045.44043126</v>
       </c>
     </row>
     <row r="6">
@@ -46825,7 +46843,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-19)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-19 (actualización 2026-07-20)</t>
         </is>
       </c>
     </row>
@@ -47152,7 +47170,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN4" s="25" t="n">
-        <v>235930884.45</v>
+        <v>235975601.38</v>
       </c>
     </row>
     <row r="5">
@@ -47266,7 +47284,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN5" s="25" t="n">
-        <v>684327181.79</v>
+        <v>684487486.2</v>
       </c>
     </row>
     <row r="6">
@@ -47608,7 +47626,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-07-19 (actualización 2026-07-19).</t>
+          <t>datos al 2026-07-19 (actualización 2026-07-20).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-07-26
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-25)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AN4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AN5</f>
@@ -3166,7 +3166,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN2" t="n">
-        <v>232795736.51</v>
+        <v>232830205.91</v>
       </c>
     </row>
     <row r="3">
@@ -3275,7 +3275,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN3" t="n">
-        <v>685290091.4299999</v>
+        <v>685450980.4400001</v>
       </c>
     </row>
     <row r="4">
@@ -3520,7 +3520,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>232795736.51</v>
+        <v>232830205.91</v>
       </c>
     </row>
     <row r="12">
@@ -3539,7 +3539,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>685290091.4299999</v>
+        <v>685450980.4400001</v>
       </c>
     </row>
     <row r="13">
@@ -3917,7 +3917,7 @@
         <v>0.003825</v>
       </c>
       <c r="AN20" t="n">
-        <v>0.003072</v>
+        <v>0.003205</v>
       </c>
     </row>
     <row r="21">
@@ -4026,7 +4026,7 @@
         <v>-3e-06</v>
       </c>
       <c r="AN21" t="n">
-        <v>0.005653</v>
+        <v>0.005889</v>
       </c>
     </row>
     <row r="22">
@@ -4252,7 +4252,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-25) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-25)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26)</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-25) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5833,6 +5833,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46228</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.17981841</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>232830205.91</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1046.91200796</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>685450980.4400001</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1224.40657971</v>
@@ -46417,7 +46435,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-25)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26)</t>
         </is>
       </c>
     </row>
@@ -46744,7 +46762,7 @@
         <v>1.17604869</v>
       </c>
       <c r="AN4" s="24" t="n">
-        <v>1.17966136</v>
+        <v>1.17981841</v>
       </c>
     </row>
     <row r="5">
@@ -46858,7 +46876,7 @@
         <v>1040.78324635</v>
       </c>
       <c r="AN5" s="24" t="n">
-        <v>1046.66627684</v>
+        <v>1046.91200796</v>
       </c>
     </row>
     <row r="6">
@@ -47229,7 +47247,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-25)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26)</t>
         </is>
       </c>
     </row>
@@ -47556,7 +47574,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN4" s="25" t="n">
-        <v>232795736.51</v>
+        <v>232830205.91</v>
       </c>
     </row>
     <row r="5">
@@ -47670,7 +47688,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN5" s="25" t="n">
-        <v>685290091.4299999</v>
+        <v>685450980.4400001</v>
       </c>
     </row>
     <row r="6">
@@ -48012,7 +48030,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-07-26 (actualización 2026-07-25).</t>
+          <t>datos al 2026-07-26 (actualización 2026-07-26).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-07-27
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-27)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AN4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AN5</f>
@@ -3166,7 +3166,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN2" t="n">
-        <v>232830205.91</v>
+        <v>232859570.14</v>
       </c>
     </row>
     <row r="3">
@@ -3275,7 +3275,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN3" t="n">
-        <v>685450980.4400001</v>
+        <v>685611337.14</v>
       </c>
     </row>
     <row r="4">
@@ -3520,7 +3520,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>232830205.91</v>
+        <v>232859570.14</v>
       </c>
     </row>
     <row r="12">
@@ -3539,7 +3539,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>685450980.4400001</v>
+        <v>685611337.14</v>
       </c>
     </row>
     <row r="13">
@@ -3917,7 +3917,7 @@
         <v>0.003825</v>
       </c>
       <c r="AN20" t="n">
-        <v>0.003205</v>
+        <v>0.003339</v>
       </c>
     </row>
     <row r="21">
@@ -4026,7 +4026,7 @@
         <v>-3e-06</v>
       </c>
       <c r="AN21" t="n">
-        <v>0.005889</v>
+        <v>0.006124</v>
       </c>
     </row>
     <row r="22">
@@ -4252,7 +4252,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-27) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-27)</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5656,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-27) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5792,6 +5792,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46229</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.17997541</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>232859570.14</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1047.15692606</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>685611337.14</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1224.64851432</v>
@@ -46435,7 +46453,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-27)</t>
         </is>
       </c>
     </row>
@@ -46762,7 +46780,7 @@
         <v>1.17604869</v>
       </c>
       <c r="AN4" s="24" t="n">
-        <v>1.17981841</v>
+        <v>1.17997541</v>
       </c>
     </row>
     <row r="5">
@@ -46876,7 +46894,7 @@
         <v>1040.78324635</v>
       </c>
       <c r="AN5" s="24" t="n">
-        <v>1046.91200796</v>
+        <v>1047.15692606</v>
       </c>
     </row>
     <row r="6">
@@ -47247,7 +47265,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-26)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-07-26 (actualización 2026-07-27)</t>
         </is>
       </c>
     </row>
@@ -47574,7 +47592,7 @@
         <v>218677379.7</v>
       </c>
       <c r="AN4" s="25" t="n">
-        <v>232830205.91</v>
+        <v>232859570.14</v>
       </c>
     </row>
     <row r="5">
@@ -47688,7 +47706,7 @@
         <v>681438259.58</v>
       </c>
       <c r="AN5" s="25" t="n">
-        <v>685450980.4400001</v>
+        <v>685611337.14</v>
       </c>
     </row>
     <row r="6">
@@ -48030,7 +48048,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-07-26 (actualización 2026-07-26).</t>
+          <t>datos al 2026-07-26 (actualización 2026-07-27).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-02
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-01)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02)</t>
         </is>
       </c>
     </row>
@@ -2607,14 +2607,14 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
         <v/>
       </c>
       <c r="H4" s="6" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I4" s="11">
         <f>E4/D4-1</f>
@@ -2647,14 +2647,14 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
         <v/>
       </c>
       <c r="H5" s="6" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I5" s="11">
         <f>E5/D5-1</f>
@@ -3173,6 +3173,9 @@
       <c r="AN2" t="n">
         <v>232122826.53</v>
       </c>
+      <c r="AO2" t="n">
+        <v>232173481.16</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3282,6 +3285,9 @@
       <c r="AN3" t="n">
         <v>686254480.35</v>
       </c>
+      <c r="AO3" t="n">
+        <v>686415182.6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3536,6 +3542,9 @@
       <c r="D11" t="n">
         <v>153562219.77</v>
       </c>
+      <c r="E11" t="n">
+        <v>232173481.16</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3552,6 +3561,9 @@
       <c r="D12" t="n">
         <v>673127647.97</v>
       </c>
+      <c r="E12" t="n">
+        <v>686415182.6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3935,6 +3947,9 @@
       <c r="AN20" t="n">
         <v>0.003993</v>
       </c>
+      <c r="AO20" t="n">
+        <v>0.000133</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4043,6 +4058,9 @@
       </c>
       <c r="AN21" t="n">
         <v>0.007068</v>
+      </c>
+      <c r="AO21" t="n">
+        <v>0.000234</v>
       </c>
     </row>
     <row r="22">
@@ -4280,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-01) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4404,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-01)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02)</t>
         </is>
       </c>
     </row>
@@ -4777,7 +4795,10 @@
         <f>IFERROR(IF(OR('Valor cuota (fin de mes)'!AN4="",'Valor cuota (fin de mes)'!AM4=""),"",'Valor cuota (fin de mes)'!AN4/'Valor cuota (fin de mes)'!AM4-1),"")</f>
         <v/>
       </c>
-      <c r="AO4" s="18" t="n"/>
+      <c r="AO4" s="17">
+        <f>IFERROR(IF(OR('Valor cuota (fin de mes)'!AO4="",'Valor cuota (fin de mes)'!AN4=""),"",'Valor cuota (fin de mes)'!AO4/'Valor cuota (fin de mes)'!AN4-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -4926,7 +4947,10 @@
         <f>IFERROR(IF(OR('Valor cuota (fin de mes)'!AN5="",'Valor cuota (fin de mes)'!AM5=""),"",'Valor cuota (fin de mes)'!AN5/'Valor cuota (fin de mes)'!AM5-1),"")</f>
         <v/>
       </c>
-      <c r="AO5" s="18" t="n"/>
+      <c r="AO5" s="17">
+        <f>IFERROR(IF(OR('Valor cuota (fin de mes)'!AO5="",'Valor cuota (fin de mes)'!AN5=""),"",'Valor cuota (fin de mes)'!AO5/'Valor cuota (fin de mes)'!AN5-1),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -5383,7 +5407,10 @@
         <f>'Rendimiento mensual'!AG4</f>
         <v/>
       </c>
-      <c r="E4" s="18" t="n"/>
+      <c r="E4" s="17">
+        <f>'Rendimiento mensual'!AO4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -5403,7 +5430,10 @@
         <f>'Rendimiento mensual'!AG5</f>
         <v/>
       </c>
-      <c r="E5" s="18" t="n"/>
+      <c r="E5" s="17">
+        <f>'Rendimiento mensual'!AO5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -5557,7 +5587,10 @@
         <f>IFERROR('Valor cuota (fin de mes)'!AG4/'Valor cuota (fin de mes)'!U4-1,"")</f>
         <v/>
       </c>
-      <c r="E4" s="18" t="n"/>
+      <c r="E4" s="17">
+        <f>IFERROR('Valor cuota (fin de mes)'!AO4/'Valor cuota (fin de mes)'!AG4-1,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -5577,7 +5610,10 @@
         <f>IFERROR('Valor cuota (fin de mes)'!AG5/'Valor cuota (fin de mes)'!U5-1,"")</f>
         <v/>
       </c>
-      <c r="E5" s="18" t="n"/>
+      <c r="E5" s="17">
+        <f>IFERROR('Valor cuota (fin de mes)'!AO5/'Valor cuota (fin de mes)'!AG5-1,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -5696,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-01) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -6037,6 +6073,24 @@
     <row r="10">
       <c r="A10" s="20" t="n">
         <v>46235</v>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>1.18090183</v>
+      </c>
+      <c r="C10" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>232173481.16</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>1048.38466589</v>
+      </c>
+      <c r="F10" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <v>686415182.6</v>
       </c>
       <c r="H10" s="21" t="n">
         <v>1226.00640372</v>
@@ -47035,7 +47089,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-01)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02)</t>
         </is>
       </c>
     </row>
@@ -47369,7 +47423,9 @@
       <c r="AN4" s="24" t="n">
         <v>1.18074522</v>
       </c>
-      <c r="AO4" s="18" t="n"/>
+      <c r="AO4" s="24" t="n">
+        <v>1.18090183</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -47484,7 +47540,9 @@
       <c r="AN5" s="24" t="n">
         <v>1048.13922001</v>
       </c>
-      <c r="AO5" s="18" t="n"/>
+      <c r="AO5" s="24" t="n">
+        <v>1048.38466589</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -47867,7 +47925,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-01)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02)</t>
         </is>
       </c>
     </row>
@@ -48201,7 +48259,9 @@
       <c r="AN4" s="25" t="n">
         <v>232122826.53</v>
       </c>
-      <c r="AO4" s="18" t="n"/>
+      <c r="AO4" s="25" t="n">
+        <v>232173481.16</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -48316,7 +48376,9 @@
       <c r="AN5" s="25" t="n">
         <v>686254480.35</v>
       </c>
-      <c r="AO5" s="18" t="n"/>
+      <c r="AO5" s="25" t="n">
+        <v>686415182.6</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -48669,7 +48731,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-06 (actualización 2026-08-01).</t>
+          <t>datos al 2026-08-06 (actualización 2026-08-02).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-03
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
@@ -3174,7 +3174,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>232173481.16</v>
+        <v>232208042.23</v>
       </c>
     </row>
     <row r="3">
@@ -3286,7 +3286,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO3" t="n">
-        <v>686415182.6</v>
+        <v>686576271.5700001</v>
       </c>
     </row>
     <row r="4">
@@ -3543,7 +3543,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>232173481.16</v>
+        <v>232208042.23</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +3562,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>686415182.6</v>
+        <v>686576271.5700001</v>
       </c>
     </row>
     <row r="13">
@@ -3948,7 +3948,7 @@
         <v>0.003993</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.000133</v>
+        <v>0.000265</v>
       </c>
     </row>
     <row r="21">
@@ -4060,7 +4060,7 @@
         <v>0.007068</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.000234</v>
+        <v>0.000469</v>
       </c>
     </row>
     <row r="22">
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -6032,6 +6032,24 @@
     <row r="9">
       <c r="A9" s="20" t="n">
         <v>46236</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>1.18105848</v>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>232208042.23</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>1048.6307024</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G9" s="23" t="n">
+        <v>686576271.5700001</v>
       </c>
       <c r="H9" s="21" t="n">
         <v>1226.16853397</v>
@@ -47089,7 +47107,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03)</t>
         </is>
       </c>
     </row>
@@ -47424,7 +47442,7 @@
         <v>1.18074522</v>
       </c>
       <c r="AO4" s="24" t="n">
-        <v>1.18090183</v>
+        <v>1.18105848</v>
       </c>
     </row>
     <row r="5">
@@ -47541,7 +47559,7 @@
         <v>1048.13922001</v>
       </c>
       <c r="AO5" s="24" t="n">
-        <v>1048.38466589</v>
+        <v>1048.6307024</v>
       </c>
     </row>
     <row r="6">
@@ -47925,7 +47943,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-02)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03)</t>
         </is>
       </c>
     </row>
@@ -48260,7 +48278,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO4" s="25" t="n">
-        <v>232173481.16</v>
+        <v>232208042.23</v>
       </c>
     </row>
     <row r="5">
@@ -48377,7 +48395,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO5" s="25" t="n">
-        <v>686415182.6</v>
+        <v>686576271.5700001</v>
       </c>
     </row>
     <row r="6">
@@ -48731,7 +48749,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-06 (actualización 2026-08-02).</t>
+          <t>datos al 2026-08-06 (actualización 2026-08-03).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-04
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46236</v>
+        <v>46240</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46236</v>
+        <v>46240</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
@@ -3174,7 +3174,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>232208042.23</v>
+        <v>233333451.63</v>
       </c>
     </row>
     <row r="3">
@@ -3286,7 +3286,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO3" t="n">
-        <v>686576271.5700001</v>
+        <v>687218908.5599999</v>
       </c>
     </row>
     <row r="4">
@@ -3543,7 +3543,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>232208042.23</v>
+        <v>233333451.63</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +3562,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>686576271.5700001</v>
+        <v>687218908.5599999</v>
       </c>
     </row>
     <row r="13">
@@ -3948,7 +3948,7 @@
         <v>0.003993</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.000265</v>
+        <v>0.000794</v>
       </c>
     </row>
     <row r="21">
@@ -4060,7 +4060,7 @@
         <v>0.007068</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.000469</v>
+        <v>0.001405</v>
       </c>
     </row>
     <row r="22">
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5869,6 +5869,24 @@
       <c r="A5" s="20" t="n">
         <v>46240</v>
       </c>
+      <c r="B5" s="21" t="n">
+        <v>1.18168246</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000132</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>233333451.63</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1049.61222319</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000233</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>687218908.5599999</v>
+      </c>
       <c r="H5" s="21" t="n">
         <v>1226.81701032</v>
       </c>
@@ -5910,6 +5928,24 @@
       <c r="A6" s="20" t="n">
         <v>46239</v>
       </c>
+      <c r="B6" s="21" t="n">
+        <v>1.18152629</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000132</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>233302614.27</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1049.36721863</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>687058495.26</v>
+      </c>
       <c r="H6" s="21" t="n">
         <v>1226.65489793</v>
       </c>
@@ -5951,6 +5987,24 @@
       <c r="A7" s="20" t="n">
         <v>46238</v>
       </c>
+      <c r="B7" s="21" t="n">
+        <v>1.18137009</v>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>0.000132</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>233271771.14</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>1049.12090227</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <v>686897223.0700001</v>
+      </c>
       <c r="H7" s="21" t="n">
         <v>1226.49278108</v>
       </c>
@@ -5991,6 +6045,24 @@
     <row r="8">
       <c r="A8" s="20" t="n">
         <v>46237</v>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>1.18121388</v>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>0.000132</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>233240926.77</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>1048.8746436</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>0.000233</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>686735988.65</v>
       </c>
       <c r="H8" s="21" t="n">
         <v>1226.33065976</v>
@@ -47107,7 +47179,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04)</t>
         </is>
       </c>
     </row>
@@ -47442,7 +47514,7 @@
         <v>1.18074522</v>
       </c>
       <c r="AO4" s="24" t="n">
-        <v>1.18105848</v>
+        <v>1.18168246</v>
       </c>
     </row>
     <row r="5">
@@ -47559,7 +47631,7 @@
         <v>1048.13922001</v>
       </c>
       <c r="AO5" s="24" t="n">
-        <v>1048.6307024</v>
+        <v>1049.61222319</v>
       </c>
     </row>
     <row r="6">
@@ -47943,7 +48015,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-03)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04)</t>
         </is>
       </c>
     </row>
@@ -48278,7 +48350,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO4" s="25" t="n">
-        <v>232208042.23</v>
+        <v>233333451.63</v>
       </c>
     </row>
     <row r="5">
@@ -48395,7 +48467,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO5" s="25" t="n">
-        <v>686576271.5700001</v>
+        <v>687218908.5599999</v>
       </c>
     </row>
     <row r="6">
@@ -48749,7 +48821,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-06 (actualización 2026-08-03).</t>
+          <t>datos al 2026-08-06 (actualización 2026-08-04).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-05
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05)</t>
         </is>
       </c>
     </row>
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -47179,7 +47179,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05)</t>
         </is>
       </c>
     </row>
@@ -48015,7 +48015,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-04)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05)</t>
         </is>
       </c>
     </row>
@@ -48821,7 +48821,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-06 (actualización 2026-08-04).</t>
+          <t>datos al 2026-08-06 (actualización 2026-08-05).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-06
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06)</t>
         </is>
       </c>
     </row>
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -47179,7 +47179,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06)</t>
         </is>
       </c>
     </row>
@@ -48015,7 +48015,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06)</t>
         </is>
       </c>
     </row>
@@ -48821,7 +48821,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-06 (actualización 2026-08-05).</t>
+          <t>datos al 2026-08-06 (actualización 2026-08-06).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-07
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-07)</t>
         </is>
       </c>
     </row>
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-07) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-07)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-07) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -47179,7 +47179,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-07)</t>
         </is>
       </c>
     </row>
@@ -48015,7 +48015,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-06)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-06 (actualización 2026-08-07)</t>
         </is>
       </c>
     </row>
@@ -48821,7 +48821,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-06 (actualización 2026-08-06).</t>
+          <t>datos al 2026-08-06 (actualización 2026-08-07).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-09
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-08)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
@@ -3174,7 +3174,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>232868106.07</v>
+        <v>232888145.18</v>
       </c>
     </row>
     <row r="3">
@@ -3286,7 +3286,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO3" t="n">
-        <v>687380344.8</v>
+        <v>687541707.0700001</v>
       </c>
     </row>
     <row r="4">
@@ -3543,7 +3543,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>232868106.07</v>
+        <v>232888145.18</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +3562,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>687380344.8</v>
+        <v>687541707.0700001</v>
       </c>
     </row>
     <row r="13">
@@ -3948,7 +3948,7 @@
         <v>0.003993</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.000927</v>
+        <v>0.00106</v>
       </c>
     </row>
     <row r="21">
@@ -4060,7 +4060,7 @@
         <v>0.007068</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.001641</v>
+        <v>0.001876</v>
       </c>
     </row>
     <row r="22">
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-08) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-08)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-08) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5909,6 +5909,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46242</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.18199707</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>232888145.18</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1050.10524405</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>687541707.0700001</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1227.14122169</v>
@@ -47320,7 +47338,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-08)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09)</t>
         </is>
       </c>
     </row>
@@ -47655,7 +47673,7 @@
         <v>1.18074522</v>
       </c>
       <c r="AO4" s="24" t="n">
-        <v>1.18184029</v>
+        <v>1.18199707</v>
       </c>
     </row>
     <row r="5">
@@ -47772,7 +47790,7 @@
         <v>1048.13922001</v>
       </c>
       <c r="AO5" s="24" t="n">
-        <v>1049.85879011</v>
+        <v>1050.10524405</v>
       </c>
     </row>
     <row r="6">
@@ -48156,7 +48174,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-08)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09)</t>
         </is>
       </c>
     </row>
@@ -48491,7 +48509,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO4" s="25" t="n">
-        <v>232868106.07</v>
+        <v>232888145.18</v>
       </c>
     </row>
     <row r="5">
@@ -48608,7 +48626,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO5" s="25" t="n">
-        <v>687380344.8</v>
+        <v>687541707.0700001</v>
       </c>
     </row>
     <row r="6">
@@ -48962,7 +48980,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-09 (actualización 2026-08-08).</t>
+          <t>datos al 2026-08-09 (actualización 2026-08-09).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-10
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-10)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
@@ -3174,7 +3174,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>232888145.18</v>
+        <v>232927883.49</v>
       </c>
     </row>
     <row r="3">
@@ -3286,7 +3286,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO3" t="n">
-        <v>687541707.0700001</v>
+        <v>687703148.23</v>
       </c>
     </row>
     <row r="4">
@@ -3543,7 +3543,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>232888145.18</v>
+        <v>232927883.49</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +3562,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>687541707.0700001</v>
+        <v>687703148.23</v>
       </c>
     </row>
     <row r="13">
@@ -3948,7 +3948,7 @@
         <v>0.003993</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.00106</v>
+        <v>0.001193</v>
       </c>
     </row>
     <row r="21">
@@ -4060,7 +4060,7 @@
         <v>0.007068</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.001876</v>
+        <v>0.002111</v>
       </c>
     </row>
     <row r="22">
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-10) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-10)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-10) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5868,6 +5868,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46243</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.18215391</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000133</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>232927883.49</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1050.35181849</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000235</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>687703148.23</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1227.30332068</v>
@@ -47338,7 +47356,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-10)</t>
         </is>
       </c>
     </row>
@@ -47673,7 +47691,7 @@
         <v>1.18074522</v>
       </c>
       <c r="AO4" s="24" t="n">
-        <v>1.18199707</v>
+        <v>1.18215391</v>
       </c>
     </row>
     <row r="5">
@@ -47790,7 +47808,7 @@
         <v>1048.13922001</v>
       </c>
       <c r="AO5" s="24" t="n">
-        <v>1050.10524405</v>
+        <v>1050.35181849</v>
       </c>
     </row>
     <row r="6">
@@ -48174,7 +48192,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-09)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-09 (actualización 2026-08-10)</t>
         </is>
       </c>
     </row>
@@ -48509,7 +48527,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO4" s="25" t="n">
-        <v>232888145.18</v>
+        <v>232927883.49</v>
       </c>
     </row>
     <row r="5">
@@ -48626,7 +48644,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO5" s="25" t="n">
-        <v>687541707.0700001</v>
+        <v>687703148.23</v>
       </c>
     </row>
     <row r="6">
@@ -48980,7 +48998,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-09 (actualización 2026-08-09).</t>
+          <t>datos al 2026-08-09 (actualización 2026-08-10).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-16
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-15)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
@@ -3174,7 +3174,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>237170013.12</v>
+        <v>237222737.87</v>
       </c>
     </row>
     <row r="3">
@@ -3286,7 +3286,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO3" t="n">
-        <v>688511704.1</v>
+        <v>688672418.4299999</v>
       </c>
     </row>
     <row r="4">
@@ -3543,7 +3543,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>237170013.12</v>
+        <v>237222737.87</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +3562,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>688511704.1</v>
+        <v>688672418.4299999</v>
       </c>
     </row>
     <row r="13">
@@ -3948,7 +3948,7 @@
         <v>0.003993</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.001855</v>
+        <v>0.001986</v>
       </c>
     </row>
     <row r="21">
@@ -4060,7 +4060,7 @@
         <v>0.007068</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.003289</v>
+        <v>0.003523</v>
       </c>
     </row>
     <row r="22">
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-15) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-15)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-15) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5909,6 +5909,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46249</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.18308997</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000131</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>237222737.87</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1051.832217</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000233</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>688672418.4299999</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1228.28943226</v>
@@ -47733,7 +47751,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-15)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16)</t>
         </is>
       </c>
     </row>
@@ -48068,7 +48086,7 @@
         <v>1.18074522</v>
       </c>
       <c r="AO4" s="24" t="n">
-        <v>1.18293496</v>
+        <v>1.18308997</v>
       </c>
     </row>
     <row r="5">
@@ -48185,7 +48203,7 @@
         <v>1048.13922001</v>
       </c>
       <c r="AO5" s="24" t="n">
-        <v>1051.58675268</v>
+        <v>1051.832217</v>
       </c>
     </row>
     <row r="6">
@@ -48569,7 +48587,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-15)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16)</t>
         </is>
       </c>
     </row>
@@ -48904,7 +48922,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO4" s="25" t="n">
-        <v>237170013.12</v>
+        <v>237222737.87</v>
       </c>
     </row>
     <row r="5">
@@ -49021,7 +49039,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO5" s="25" t="n">
-        <v>688511704.1</v>
+        <v>688672418.4299999</v>
       </c>
     </row>
     <row r="6">
@@ -49375,7 +49393,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-16 (actualización 2026-08-15).</t>
+          <t>datos al 2026-08-16 (actualización 2026-08-16).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-17
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-17)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
@@ -3174,7 +3174,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>237222737.87</v>
+        <v>237259321.85</v>
       </c>
     </row>
     <row r="3">
@@ -3286,7 +3286,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO3" t="n">
-        <v>688672418.4299999</v>
+        <v>688833057.8200001</v>
       </c>
     </row>
     <row r="4">
@@ -3543,7 +3543,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>237222737.87</v>
+        <v>237259321.85</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +3562,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>688672418.4299999</v>
+        <v>688833057.8200001</v>
       </c>
     </row>
     <row r="13">
@@ -3948,7 +3948,7 @@
         <v>0.003993</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.001986</v>
+        <v>0.002117</v>
       </c>
     </row>
     <row r="21">
@@ -4060,7 +4060,7 @@
         <v>0.007068</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.003523</v>
+        <v>0.003757</v>
       </c>
     </row>
     <row r="22">
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-17) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-17)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-17) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5868,6 +5868,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46250</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.18324438</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000131</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>237259321.85</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1052.07756686</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000233</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>688833057.8200001</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1228.45547997</v>
@@ -47751,7 +47769,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-17)</t>
         </is>
       </c>
     </row>
@@ -48086,7 +48104,7 @@
         <v>1.18074522</v>
       </c>
       <c r="AO4" s="24" t="n">
-        <v>1.18308997</v>
+        <v>1.18324438</v>
       </c>
     </row>
     <row r="5">
@@ -48203,7 +48221,7 @@
         <v>1048.13922001</v>
       </c>
       <c r="AO5" s="24" t="n">
-        <v>1051.832217</v>
+        <v>1052.07756686</v>
       </c>
     </row>
     <row r="6">
@@ -48587,7 +48605,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-16)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-16 (actualización 2026-08-17)</t>
         </is>
       </c>
     </row>
@@ -48922,7 +48940,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO4" s="25" t="n">
-        <v>237222737.87</v>
+        <v>237259321.85</v>
       </c>
     </row>
     <row r="5">
@@ -49039,7 +49057,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO5" s="25" t="n">
-        <v>688672418.4299999</v>
+        <v>688833057.8200001</v>
       </c>
     </row>
     <row r="6">
@@ -49393,7 +49411,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-16 (actualización 2026-08-16).</t>
+          <t>datos al 2026-08-16 (actualización 2026-08-17).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-23
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-22)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
@@ -3174,7 +3174,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>244011559.25</v>
+        <v>244045292.1</v>
       </c>
     </row>
     <row r="3">
@@ -3286,7 +3286,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO3" t="n">
-        <v>689617522.99</v>
+        <v>689778497.79</v>
       </c>
     </row>
     <row r="4">
@@ -3543,7 +3543,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>244011559.25</v>
+        <v>244045292.1</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +3562,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>689617522.99</v>
+        <v>689778497.79</v>
       </c>
     </row>
     <row r="13">
@@ -3948,7 +3948,7 @@
         <v>0.003993</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.002725</v>
+        <v>0.002856</v>
       </c>
     </row>
     <row r="21">
@@ -4060,7 +4060,7 @@
         <v>0.007068</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.004901</v>
+        <v>0.005135</v>
       </c>
     </row>
     <row r="22">
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-22) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-22)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-22) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5909,6 +5909,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46256</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.1841176</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000131</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>244045292.1</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1053.52156868</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000233</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>689778497.79</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1229.40460714</v>
@@ -48146,7 +48164,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-22)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23)</t>
         </is>
       </c>
     </row>
@@ -48481,7 +48499,7 @@
         <v>1.18074522</v>
       </c>
       <c r="AO4" s="24" t="n">
-        <v>1.18396283</v>
+        <v>1.1841176</v>
       </c>
     </row>
     <row r="5">
@@ -48598,7 +48616,7 @@
         <v>1048.13922001</v>
       </c>
       <c r="AO5" s="24" t="n">
-        <v>1053.27570653</v>
+        <v>1053.52156868</v>
       </c>
     </row>
     <row r="6">
@@ -48982,7 +49000,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-22)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23)</t>
         </is>
       </c>
     </row>
@@ -49317,7 +49335,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO4" s="25" t="n">
-        <v>244011559.25</v>
+        <v>244045292.1</v>
       </c>
     </row>
     <row r="5">
@@ -49434,7 +49452,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO5" s="25" t="n">
-        <v>689617522.99</v>
+        <v>689778497.79</v>
       </c>
     </row>
     <row r="6">
@@ -49788,7 +49806,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-23 (actualización 2026-08-22).</t>
+          <t>datos al 2026-08-23 (actualización 2026-08-23).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-24
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-24)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
@@ -3174,7 +3174,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>244045292.1</v>
+        <v>244066799.75</v>
       </c>
     </row>
     <row r="3">
@@ -3286,7 +3286,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO3" t="n">
-        <v>689778497.79</v>
+        <v>689939478.8099999</v>
       </c>
     </row>
     <row r="4">
@@ -3543,7 +3543,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>244045292.1</v>
+        <v>244066799.75</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +3562,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>689778497.79</v>
+        <v>689939478.8099999</v>
       </c>
     </row>
     <row r="13">
@@ -3948,7 +3948,7 @@
         <v>0.003993</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.002856</v>
+        <v>0.002982</v>
       </c>
     </row>
     <row r="21">
@@ -4060,7 +4060,7 @@
         <v>0.007068</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.005135</v>
+        <v>0.00537</v>
       </c>
     </row>
     <row r="22">
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-24) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-24)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-24) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5868,6 +5868,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46257</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.18426655</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000126</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>244066799.75</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1053.76744033</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000233</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>689939478.8099999</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1229.56183678</v>
@@ -48164,7 +48182,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-24)</t>
         </is>
       </c>
     </row>
@@ -48499,7 +48517,7 @@
         <v>1.18074522</v>
       </c>
       <c r="AO4" s="24" t="n">
-        <v>1.1841176</v>
+        <v>1.18426655</v>
       </c>
     </row>
     <row r="5">
@@ -48616,7 +48634,7 @@
         <v>1048.13922001</v>
       </c>
       <c r="AO5" s="24" t="n">
-        <v>1053.52156868</v>
+        <v>1053.76744033</v>
       </c>
     </row>
     <row r="6">
@@ -49000,7 +49018,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-23)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-23 (actualización 2026-08-24)</t>
         </is>
       </c>
     </row>
@@ -49335,7 +49353,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO4" s="25" t="n">
-        <v>244045292.1</v>
+        <v>244066799.75</v>
       </c>
     </row>
     <row r="5">
@@ -49452,7 +49470,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO5" s="25" t="n">
-        <v>689778497.79</v>
+        <v>689939478.8099999</v>
       </c>
     </row>
     <row r="6">
@@ -49806,7 +49824,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-23 (actualización 2026-08-23).</t>
+          <t>datos al 2026-08-23 (actualización 2026-08-24).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-30
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-29)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
@@ -3174,7 +3174,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>242279491.15</v>
+        <v>242352279.56</v>
       </c>
     </row>
     <row r="3">
@@ -3286,7 +3286,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO3" t="n">
-        <v>687142609.23</v>
+        <v>687303615.23</v>
       </c>
     </row>
     <row r="4">
@@ -3543,7 +3543,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>242279491.15</v>
+        <v>242352279.56</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +3562,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>687142609.23</v>
+        <v>687303615.23</v>
       </c>
     </row>
     <row r="13">
@@ -3948,7 +3948,7 @@
         <v>0.003993</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.003628</v>
+        <v>0.003762</v>
       </c>
     </row>
     <row r="21">
@@ -4060,7 +4060,7 @@
         <v>0.007068</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.001294</v>
+        <v>0.001529</v>
       </c>
     </row>
     <row r="22">
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-29) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-29)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-29) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5909,6 +5909,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46263</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.18518669</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000134</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>242352279.56</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1049.7415985</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>687303615.23</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1238.58482289</v>
@@ -48559,7 +48577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-29)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30)</t>
         </is>
       </c>
     </row>
@@ -48894,7 +48912,7 @@
         <v>1.18074522</v>
       </c>
       <c r="AO4" s="24" t="n">
-        <v>1.18502848</v>
+        <v>1.18518669</v>
       </c>
     </row>
     <row r="5">
@@ -49011,7 +49029,7 @@
         <v>1048.13922001</v>
       </c>
       <c r="AO5" s="24" t="n">
-        <v>1049.49568869</v>
+        <v>1049.7415985</v>
       </c>
     </row>
     <row r="6">
@@ -49395,7 +49413,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-29)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30)</t>
         </is>
       </c>
     </row>
@@ -49730,7 +49748,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO4" s="25" t="n">
-        <v>242279491.15</v>
+        <v>242352279.56</v>
       </c>
     </row>
     <row r="5">
@@ -49847,7 +49865,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO5" s="25" t="n">
-        <v>687142609.23</v>
+        <v>687303615.23</v>
       </c>
     </row>
     <row r="6">
@@ -50201,7 +50219,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-30 (actualización 2026-08-29).</t>
+          <t>datos al 2026-08-30 (actualización 2026-08-30).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-08-31
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-31)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AO4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AO5</f>
@@ -3174,7 +3174,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO2" t="n">
-        <v>242352279.56</v>
+        <v>242390168.79</v>
       </c>
     </row>
     <row r="3">
@@ -3286,7 +3286,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO3" t="n">
-        <v>687303615.23</v>
+        <v>687311254.28</v>
       </c>
     </row>
     <row r="4">
@@ -3543,7 +3543,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>242352279.56</v>
+        <v>242390168.79</v>
       </c>
     </row>
     <row r="12">
@@ -3562,7 +3562,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>687303615.23</v>
+        <v>687311254.28</v>
       </c>
     </row>
     <row r="13">
@@ -3948,7 +3948,7 @@
         <v>0.003993</v>
       </c>
       <c r="AO20" t="n">
-        <v>0.003762</v>
+        <v>0.003902</v>
       </c>
     </row>
     <row r="21">
@@ -4060,7 +4060,7 @@
         <v>0.007068</v>
       </c>
       <c r="AO21" t="n">
-        <v>0.001529</v>
+        <v>0.00154</v>
       </c>
     </row>
     <row r="22">
@@ -4298,7 +4298,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-31) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-31)</t>
         </is>
       </c>
     </row>
@@ -5732,7 +5732,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-31) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5868,6 +5868,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46264</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.18535255</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.00014</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>242390168.79</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1049.75326587</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>1.1e-05</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>687311254.28</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1238.82470988</v>
@@ -48577,7 +48595,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-31)</t>
         </is>
       </c>
     </row>
@@ -48912,7 +48930,7 @@
         <v>1.18074522</v>
       </c>
       <c r="AO4" s="24" t="n">
-        <v>1.18518669</v>
+        <v>1.18535255</v>
       </c>
     </row>
     <row r="5">
@@ -49029,7 +49047,7 @@
         <v>1048.13922001</v>
       </c>
       <c r="AO5" s="24" t="n">
-        <v>1049.7415985</v>
+        <v>1049.75326587</v>
       </c>
     </row>
     <row r="6">
@@ -49413,7 +49431,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-30)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-08-30 (actualización 2026-08-31)</t>
         </is>
       </c>
     </row>
@@ -49748,7 +49766,7 @@
         <v>232122826.53</v>
       </c>
       <c r="AO4" s="25" t="n">
-        <v>242352279.56</v>
+        <v>242390168.79</v>
       </c>
     </row>
     <row r="5">
@@ -49865,7 +49883,7 @@
         <v>686254480.35</v>
       </c>
       <c r="AO5" s="25" t="n">
-        <v>687303615.23</v>
+        <v>687311254.28</v>
       </c>
     </row>
     <row r="6">
@@ -50219,7 +50237,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-08-30 (actualización 2026-08-30).</t>
+          <t>datos al 2026-08-30 (actualización 2026-08-31).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-09-06
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AP4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AP5</f>
@@ -3182,7 +3182,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP2" t="n">
-        <v>251728775.36</v>
+        <v>251810071.58</v>
       </c>
     </row>
     <row r="3">
@@ -3297,7 +3297,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP3" t="n">
-        <v>688206769.4299999</v>
+        <v>688367884.67</v>
       </c>
     </row>
     <row r="4">
@@ -3566,7 +3566,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>251728775.36</v>
+        <v>251810071.58</v>
       </c>
     </row>
     <row r="12">
@@ -3585,7 +3585,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>688206769.4299999</v>
+        <v>688367884.67</v>
       </c>
     </row>
     <row r="13">
@@ -3979,7 +3979,7 @@
         <v>0.004052</v>
       </c>
       <c r="AP20" t="n">
-        <v>0.00049</v>
+        <v>0.000617</v>
       </c>
     </row>
     <row r="21">
@@ -4094,7 +4094,7 @@
         <v>0.001774</v>
       </c>
       <c r="AP21" t="n">
-        <v>0.001069</v>
+        <v>0.001303</v>
       </c>
     </row>
     <row r="22">
@@ -4344,7 +4344,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-05) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-05) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5985,6 +5985,24 @@
     <row r="6">
       <c r="A6" s="20" t="n">
         <v>46270</v>
+      </c>
+      <c r="B6" s="21" t="n">
+        <v>1.18626189</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>0.000128</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>251810071.58</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>1051.36709249</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>688367884.67</v>
       </c>
       <c r="H6" s="21" t="n">
         <v>1239.97460535</v>
@@ -49049,7 +49067,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06)</t>
         </is>
       </c>
     </row>
@@ -49392,7 +49410,7 @@
         <v>1.18553004</v>
       </c>
       <c r="AP4" s="24" t="n">
-        <v>1.18611058</v>
+        <v>1.18626189</v>
       </c>
     </row>
     <row r="5">
@@ -49512,7 +49530,7 @@
         <v>1049.99873259</v>
       </c>
       <c r="AP5" s="24" t="n">
-        <v>1051.12101584</v>
+        <v>1051.36709249</v>
       </c>
     </row>
     <row r="6">
@@ -49909,7 +49927,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-05)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06)</t>
         </is>
       </c>
     </row>
@@ -50252,7 +50270,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP4" s="25" t="n">
-        <v>251728775.36</v>
+        <v>251810071.58</v>
       </c>
     </row>
     <row r="5">
@@ -50372,7 +50390,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP5" s="25" t="n">
-        <v>688206769.4299999</v>
+        <v>688367884.67</v>
       </c>
     </row>
     <row r="6">
@@ -50738,7 +50756,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-09-06 (actualización 2026-09-05).</t>
+          <t>datos al 2026-09-06 (actualización 2026-09-06).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática: datos al 2026-09-07
</commit_message>
<xml_diff>
--- a/hencorp.xlsx
+++ b/hencorp.xlsx
@@ -2529,7 +2529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-07)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v/>
       </c>
       <c r="F4" s="7" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="G4" s="10">
         <f>'Patrimonio (fin de mes)'!AP4</f>
@@ -2647,7 +2647,7 @@
         <v/>
       </c>
       <c r="F5" s="7" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="G5" s="10">
         <f>'Patrimonio (fin de mes)'!AP5</f>
@@ -3182,7 +3182,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP2" t="n">
-        <v>251810071.58</v>
+        <v>251916879.41</v>
       </c>
     </row>
     <row r="3">
@@ -3297,7 +3297,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP3" t="n">
-        <v>688367884.67</v>
+        <v>688529025.91</v>
       </c>
     </row>
     <row r="4">
@@ -3566,7 +3566,7 @@
         <v>153562219.77</v>
       </c>
       <c r="E11" t="n">
-        <v>251810071.58</v>
+        <v>251916879.41</v>
       </c>
     </row>
     <row r="12">
@@ -3585,7 +3585,7 @@
         <v>673127647.97</v>
       </c>
       <c r="E12" t="n">
-        <v>688367884.67</v>
+        <v>688529025.91</v>
       </c>
     </row>
     <row r="13">
@@ -3979,7 +3979,7 @@
         <v>0.004052</v>
       </c>
       <c r="AP20" t="n">
-        <v>0.000617</v>
+        <v>0.000744</v>
       </c>
     </row>
     <row r="21">
@@ -4094,7 +4094,7 @@
         <v>0.001774</v>
       </c>
       <c r="AP21" t="n">
-        <v>0.001303</v>
+        <v>0.001538</v>
       </c>
     </row>
     <row r="22">
@@ -4344,7 +4344,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-07) | una gráfica por fondo · cada una con su propio eje · se actualizan solas al crecer meses/días</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-07)</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-07) | una fila por día · lo más reciente arriba · se actualiza a diario</t>
         </is>
       </c>
     </row>
@@ -5944,6 +5944,24 @@
     <row r="5">
       <c r="A5" s="20" t="n">
         <v>46271</v>
+      </c>
+      <c r="B5" s="21" t="n">
+        <v>1.18641153</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>0.000126</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>251916879.41</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <v>1051.61320885</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0.000234</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>688529025.91</v>
       </c>
       <c r="H5" s="21" t="n">
         <v>1240.1563452</v>
@@ -49067,7 +49085,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-07)</t>
         </is>
       </c>
     </row>
@@ -49410,7 +49428,7 @@
         <v>1.18553004</v>
       </c>
       <c r="AP4" s="24" t="n">
-        <v>1.18626189</v>
+        <v>1.18641153</v>
       </c>
     </row>
     <row r="5">
@@ -49530,7 +49548,7 @@
         <v>1049.99873259</v>
       </c>
       <c r="AP5" s="24" t="n">
-        <v>1051.36709249</v>
+        <v>1051.61320885</v>
       </c>
     </row>
     <row r="6">
@@ -49927,7 +49945,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-06)</t>
+          <t>Grupo Hencorp — Gestora de Fondos | Fuente: hencorpgestora.com (Comportamiento Histórico) | datos al 2026-09-06 (actualización 2026-09-07)</t>
         </is>
       </c>
     </row>
@@ -50270,7 +50288,7 @@
         <v>246137246.86</v>
       </c>
       <c r="AP4" s="25" t="n">
-        <v>251810071.58</v>
+        <v>251916879.41</v>
       </c>
     </row>
     <row r="5">
@@ -50390,7 +50408,7 @@
         <v>687471970.1799999</v>
       </c>
       <c r="AP5" s="25" t="n">
-        <v>688367884.67</v>
+        <v>688529025.91</v>
       </c>
     </row>
     <row r="6">
@@ -50756,7 +50774,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>datos al 2026-09-06 (actualización 2026-09-06).</t>
+          <t>datos al 2026-09-06 (actualización 2026-09-07).</t>
         </is>
       </c>
     </row>

</xml_diff>